<commit_message>
chore(vas): Duncan's wording for the prepaid electricity labels
Replaces the placeholder phrasing with his own, and applied to the crosstab
config files in the project folder.

Two things his version does better. 'Average ... value per transaction' says on
its face that the figure is an average, which is the statistic that has been
causing the reconciliation confusion — spend/transactions per person, not total
spend over total transactions. And '(for everyone)' states the Total view
explicitly rather than leaving it as the unmarked case.

Note: this now diverges from reader_label() in build_vas_reporting_config.py,
which still writes 'Prepaid electricity — transactions a month' for the section
reports. Same measures, two wordings, until one is brought to the other.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/vas/vas_report_labels.xlsx
+++ b/modules/vas/vas_report_labels.xlsx
@@ -1,205 +1,212 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr date1904="false"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/duncan/Dev/Turas/modules/vas/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB585A9E-2039-1F44-B01B-6F13E1A39067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13125" windowHeight="6105" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="19620" windowHeight="15220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Labels" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Labels" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="60">
-  <si>
-    <t xml:space="preserve">question_code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">question_text</t>
-  </si>
-  <si>
-    <t xml:space="preserve">note</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Age</t>
-  </si>
-  <si>
-    <t xml:space="preserve">was: What is your age?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gender</t>
-  </si>
-  <si>
-    <t xml:space="preserve">unchanged — already reads as a label</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Race</t>
-  </si>
-  <si>
-    <t xml:space="preserve">was: Which best describes your ethnic group?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Province</t>
-  </si>
-  <si>
-    <t xml:space="preserve">was: Which province do you currently live in?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Town</t>
-  </si>
-  <si>
-    <t xml:space="preserve">coalesced from the nine per-province questions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AreaType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Type of area lived in</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matches the reporting build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Income</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Monthly household income</t>
-  </si>
-  <si>
-    <t xml:space="preserve">was: Monthly household income category?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BillPayer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Role in paying household bills</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Purchased</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buy electricity at all in last 12 months?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1. derived from transactions a month above zero, not from the screener</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PPU</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Who have you bought electricity for?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. self / other / none — the base already says who is in it</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Total_TxnPerMonth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — transactions a month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Total_MonthlySpend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — spend a month</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Total_SpendPerTxn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — value per transaction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. total — per-buyer average, see note below</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Own_TxnPerMonth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — transactions a month (for self)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. for self</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Own_MonthlySpend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — spend a month (for self)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7. for self</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Own_SpendPerTxn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — value per transaction (for self)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8. for self — per-buyer average</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Oth_TxnPerMonth</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — transactions a month (for others)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9. for others</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Oth_MonthlySpend</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — spend a month (for others)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10. for others</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PrepaidElectricity_Oth_SpendPerTxn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prepaid electricity — value per transaction (for others)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">11. for others — per-buyer average</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PPUChannelMain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Where do you buy prepaid electricity most often?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">12.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PPUOthChannel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Where else have you bought prepaid electricity?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">13. multi-column</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="60">
+  <si>
+    <t>question_code</t>
+  </si>
+  <si>
+    <t>question_text</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>Age</t>
+  </si>
+  <si>
+    <t>was: What is your age?</t>
+  </si>
+  <si>
+    <t>Gender</t>
+  </si>
+  <si>
+    <t>unchanged — already reads as a label</t>
+  </si>
+  <si>
+    <t>Race</t>
+  </si>
+  <si>
+    <t>was: Which best describes your ethnic group?</t>
+  </si>
+  <si>
+    <t>Province</t>
+  </si>
+  <si>
+    <t>was: Which province do you currently live in?</t>
+  </si>
+  <si>
+    <t>Town</t>
+  </si>
+  <si>
+    <t>coalesced from the nine per-province questions</t>
+  </si>
+  <si>
+    <t>AreaType</t>
+  </si>
+  <si>
+    <t>Type of area lived in</t>
+  </si>
+  <si>
+    <t>matches the reporting build</t>
+  </si>
+  <si>
+    <t>Income</t>
+  </si>
+  <si>
+    <t>Monthly household income</t>
+  </si>
+  <si>
+    <t>was: Monthly household income category?</t>
+  </si>
+  <si>
+    <t>BillPayer</t>
+  </si>
+  <si>
+    <t>Role in paying household bills</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Purchased</t>
+  </si>
+  <si>
+    <t>Buy electricity at all in last 12 months?</t>
+  </si>
+  <si>
+    <t>1. derived from transactions a month above zero, not from the screener</t>
+  </si>
+  <si>
+    <t>PPU</t>
+  </si>
+  <si>
+    <t>Who have you bought electricity for?</t>
+  </si>
+  <si>
+    <t>2. self / other / none — the base already says who is in it</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Total_TxnPerMonth</t>
+  </si>
+  <si>
+    <t>3. total</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Total_MonthlySpend</t>
+  </si>
+  <si>
+    <t>4. total</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Total_SpendPerTxn</t>
+  </si>
+  <si>
+    <t>5. total — per-buyer average, see note below</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Own_TxnPerMonth</t>
+  </si>
+  <si>
+    <t>6. for self</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Own_MonthlySpend</t>
+  </si>
+  <si>
+    <t>7. for self</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Own_SpendPerTxn</t>
+  </si>
+  <si>
+    <t>8. for self — per-buyer average</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Oth_TxnPerMonth</t>
+  </si>
+  <si>
+    <t>9. for others</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Oth_MonthlySpend</t>
+  </si>
+  <si>
+    <t>10. for others</t>
+  </si>
+  <si>
+    <t>PrepaidElectricity_Oth_SpendPerTxn</t>
+  </si>
+  <si>
+    <t>11. for others — per-buyer average</t>
+  </si>
+  <si>
+    <t>PPUChannelMain</t>
+  </si>
+  <si>
+    <t>Where do you buy prepaid electricity most often?</t>
+  </si>
+  <si>
+    <t>12.</t>
+  </si>
+  <si>
+    <t>PPUOthChannel</t>
+  </si>
+  <si>
+    <t>13. multi-column</t>
+  </si>
+  <si>
+    <t>Prepaid electricity transactions per month (for self)</t>
+  </si>
+  <si>
+    <t>Prepaid electricity spend per month (for self)</t>
+  </si>
+  <si>
+    <t>Prepaid electricity transactions per month (for others)</t>
+  </si>
+  <si>
+    <t>Prepaid electricity spend per month (for others)</t>
+  </si>
+  <si>
+    <t>Where else have you bought prepaid electricity in the past 12 months?</t>
+  </si>
+  <si>
+    <t>Prepaid electricity transactions per month (for everyone)</t>
+  </si>
+  <si>
+    <t>Prepaid electricity spend per month (for everyone)</t>
+  </si>
+  <si>
+    <t>Average Prepaid electricity value per transaction (for everyone)</t>
+  </si>
+  <si>
+    <t>Average Prepaid electricity value per transaction (for self)</t>
+  </si>
+  <si>
+    <t>Average Prepaid electricity value per transaction (for others)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -208,10 +215,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <b/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -242,6 +250,15 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -523,16 +540,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="40.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="54.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="62.71" hidden="0" customWidth="1"/>
+    <col min="1" max="1" width="40.6640625" customWidth="1"/>
+    <col min="2" max="2" width="54.6640625" customWidth="1"/>
+    <col min="3" max="3" width="62.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -543,7 +560,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -554,7 +571,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -565,7 +582,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -576,7 +593,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -587,7 +604,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -598,7 +615,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -609,7 +626,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -620,7 +637,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -631,7 +648,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -642,7 +659,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -653,129 +670,129 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>27</v>
       </c>
       <c r="B12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" t="s">
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13" t="s">
         <v>30</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
         <v>31</v>
       </c>
-      <c r="C13" t="s">
+      <c r="B14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="s">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
         <v>33</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B15" t="s">
+        <v>50</v>
+      </c>
+      <c r="C15" t="s">
         <v>34</v>
       </c>
-      <c r="C14" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
+      <c r="B16" t="s">
+        <v>51</v>
+      </c>
+      <c r="C16" t="s">
         <v>36</v>
       </c>
-      <c r="B15" t="s">
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
         <v>37</v>
       </c>
-      <c r="C15" t="s">
+      <c r="B17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="s">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
         <v>39</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B18" t="s">
+        <v>52</v>
+      </c>
+      <c r="C18" t="s">
         <v>40</v>
       </c>
-      <c r="C16" t="s">
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
+      <c r="B19" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" t="s">
         <v>42</v>
       </c>
-      <c r="B17" t="s">
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
         <v>43</v>
       </c>
-      <c r="C17" t="s">
+      <c r="B20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="s">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
         <v>45</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B21" t="s">
         <v>46</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C21" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="s">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
         <v>48</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B22" t="s">
+        <v>54</v>
+      </c>
+      <c r="C22" t="s">
         <v>49</v>
-      </c>
-      <c r="C19" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C20" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>54</v>
-      </c>
-      <c r="B21" t="s">
-        <v>55</v>
-      </c>
-      <c r="C21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>57</v>
-      </c>
-      <c r="B22" t="s">
-        <v>58</v>
-      </c>
-      <c r="C22" t="s">
-        <v>59</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(vas): the transactions row says what it counts, and over what period
Duncan: "Number of Prepaid Electricity transactions per month". It was a
question ("How often do you buy...?"), which is wrong twice over — nobody was
asked a monthly count, it comes off the frequency cascade; and the earlier
"in the past 12 months" wording invited a reader to take the 2.54 as a yearly
total when the bands underneath read once a week, a few times a month, once a
month.

The rule takes a Title Case category name for rows that lead with it, beside
the lowercase phrase used mid-sentence, so replication carries both.

Live block verified and the labels file diffed against the kept structure —
11 codes, no disagreement. VAS suite 564/0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/vas/vas_report_labels.xlsx
+++ b/modules/vas/vas_report_labels.xlsx
@@ -89,7 +89,7 @@
     <t xml:space="preserve">PrepaidElectricity_Total_TxnPerMonth</t>
   </si>
   <si>
-    <t xml:space="preserve">How often do you buy prepaid electricity? (all buyers)</t>
+    <t xml:space="preserve">Number of Prepaid Electricity transactions per month (all buyers)</t>
   </si>
   <si>
     <t xml:space="preserve">PrepaidElectricity_Total_MonthlySpend</t>
@@ -107,7 +107,7 @@
     <t xml:space="preserve">PrepaidElectricity_Own_TxnPerMonth</t>
   </si>
   <si>
-    <t xml:space="preserve">How often do you buy prepaid electricity? (for self)</t>
+    <t xml:space="preserve">Number of Prepaid Electricity transactions per month (for self)</t>
   </si>
   <si>
     <t xml:space="preserve">PrepaidElectricity_Own_MonthlySpend</t>
@@ -125,7 +125,7 @@
     <t xml:space="preserve">PrepaidElectricity_Oth_TxnPerMonth</t>
   </si>
   <si>
-    <t xml:space="preserve">How often do you buy prepaid electricity? (for others)</t>
+    <t xml:space="preserve">Number of Prepaid Electricity transactions per month (for others)</t>
   </si>
   <si>
     <t xml:space="preserve">PrepaidElectricity_Oth_MonthlySpend</t>

</xml_diff>

<commit_message>
feat(vas): the total row says all purchases, not all buyers
Duncan's call, and the reasoning is the useful part: all three measure rows sit
on BUYERS — 765, 727 and 87 of them on electricity — so the base is not what
tells them apart. Who the purchase was for is. "(all buyers)" described the
base and so distinguished nothing.

"(for everyone)" was rejected for overstating it: the base is the 765 buyers,
not the 1,026 adults, and the figures that genuinely are across every adult
live elsewhere in the reporting layer. "(Total)" was rejected because the
banner's own first column is headed Total.

Live block verified, no "all buyers" left in the structure, the config or the
labels file, and the three still agree across all 11 codes. VAS suite 564/0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/vas/vas_report_labels.xlsx
+++ b/modules/vas/vas_report_labels.xlsx
@@ -89,19 +89,19 @@
     <t xml:space="preserve">PrepaidElectricity_Total_TxnPerMonth</t>
   </si>
   <si>
-    <t xml:space="preserve">Number of Prepaid Electricity transactions per month (all buyers)</t>
+    <t xml:space="preserve">Number of Prepaid Electricity transactions per month (all purchases)</t>
   </si>
   <si>
     <t xml:space="preserve">PrepaidElectricity_Total_MonthlySpend</t>
   </si>
   <si>
-    <t xml:space="preserve">How much do you spend per month on prepaid electricity? (all buyers)</t>
+    <t xml:space="preserve">How much do you spend per month on prepaid electricity? (all purchases)</t>
   </si>
   <si>
     <t xml:space="preserve">PrepaidElectricity_Total_SpendPerTxn</t>
   </si>
   <si>
-    <t xml:space="preserve">Average prepaid electricity value per transaction (all buyers)</t>
+    <t xml:space="preserve">Average prepaid electricity value per transaction (all purchases)</t>
   </si>
   <si>
     <t xml:space="preserve">PrepaidElectricity_Own_TxnPerMonth</t>

</xml_diff>

<commit_message>
feat(vas): multi-mentions possible, and the total-used channel row says all purchases
Duncan's wording, both places: the screener reads "(multi-mentions possible)",
and the total-used channel table reads "Where do you buy prepaid electricity -
all purchases" to match the measure rows above it.

Proved the whole build runs, not just the pieces: build_turas_dataset over the
live export into a scratch folder — 1,026 respondents x 1,087 columns, the 14
occasions gaining their two channel tables, all 138 labels applied with no
unknown code, and the fresh-generation branch writing a structure and config
from scratch with 71 ratio pairs declared and all 14 raw where-else rows
hidden. The kept pair and a freshly generated one now say the same thing.

VAS suite 564/0.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/modules/vas/vas_report_labels.xlsx
+++ b/modules/vas/vas_report_labels.xlsx
@@ -143,7 +143,7 @@
     <t xml:space="preserve">PPU</t>
   </si>
   <si>
-    <t xml:space="preserve">Who have you bought electricity for? (more than one may apply)</t>
+    <t xml:space="preserve">Who have you bought electricity for? (multi-mentions possible)</t>
   </si>
   <si>
     <t xml:space="preserve">ASKED - self / other / none</t>
@@ -152,7 +152,7 @@
     <t xml:space="preserve">PPUChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy prepaid electricity - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy prepaid electricity - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">DERIVED from the most-often and where-else questions</t>
@@ -197,7 +197,7 @@
     <t xml:space="preserve">AirtimeChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy prepaid airtime - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy prepaid airtime - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">AirtimeChannelMain</t>
@@ -233,7 +233,7 @@
     <t xml:space="preserve">DataChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy prepaid data - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy prepaid data - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">DataChannelMain</t>
@@ -272,7 +272,7 @@
     <t xml:space="preserve">LottoChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy LOTTO - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy LOTTO - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">LottoChannelMain</t>
@@ -308,7 +308,7 @@
     <t xml:space="preserve">BetChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy betting vouchers - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy betting vouchers - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">BetChannelMain</t>
@@ -362,7 +362,7 @@
     <t xml:space="preserve">VoucherChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy digital vouchers - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy digital vouchers - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">VoucherChannelMain</t>
@@ -407,7 +407,7 @@
     <t xml:space="preserve">DomSendChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you send domestic money transfers from - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you send domestic money transfers from - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">DomSendChannelMain</t>
@@ -443,7 +443,7 @@
     <t xml:space="preserve">DomRcvChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you collect domestic money transfers - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you collect domestic money transfers - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">DomRcvChannelMain</t>
@@ -485,7 +485,7 @@
     <t xml:space="preserve">IntlSendChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you pay for international money transfers - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you pay for international money transfers - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">IntlSendChannelMain</t>
@@ -530,7 +530,7 @@
     <t xml:space="preserve">FlightChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy flight tickets - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy flight tickets - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">FlightChannelMain</t>
@@ -566,7 +566,7 @@
     <t xml:space="preserve">LDBusChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy long distance bus tickets - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy long distance bus tickets - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">LDBusChannelMain</t>
@@ -602,7 +602,7 @@
     <t xml:space="preserve">SDBusChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy short distance bus tickets - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy short distance bus tickets - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">SDBusChannelMain</t>
@@ -647,7 +647,7 @@
     <t xml:space="preserve">BillChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you pay bills - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you pay bills - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">BillChannelMain</t>
@@ -770,7 +770,7 @@
     <t xml:space="preserve">EventChannelEver</t>
   </si>
   <si>
-    <t xml:space="preserve">Where do you buy event tickets - all channels used, most often or also?</t>
+    <t xml:space="preserve">Where do you buy event tickets - all purchases</t>
   </si>
   <si>
     <t xml:space="preserve">EventChannelMain</t>

</xml_diff>